<commit_message>
No change in max sng for riding & trot/race horses
</commit_message>
<xml_diff>
--- a/scenarios/REC_HORSES.xlsx
+++ b/scenarios/REC_HORSES.xlsx
@@ -4,10 +4,10 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12180" activeTab="1"/>
   </bookViews>
   <sheets>
-    <sheet name="HorseHerd" sheetId="1" r:id="rId1"/>
+    <sheet name="HorseHerd(dropped)" sheetId="1" r:id="rId1"/>
     <sheet name="FeedMgmt" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="27">
   <si>
     <t>riding horses</t>
   </si>
@@ -95,6 +95,12 @@
   </si>
   <si>
     <t>trotters and racehorses</t>
+  </si>
+  <si>
+    <t>low-performing horses</t>
+  </si>
+  <si>
+    <t>medium-performing horses</t>
   </si>
 </sst>
 </file>
@@ -521,7 +527,7 @@
         <v>11</v>
       </c>
       <c r="F4" s="2">
-        <f t="shared" ref="F4:F17" si="0">SUM(J4:J5)-F5</f>
+        <f t="shared" ref="F4" si="0">SUM(J4:J5)-F5</f>
         <v>55.199999599999998</v>
       </c>
       <c r="H4">
@@ -548,7 +554,7 @@
         <v>11</v>
       </c>
       <c r="F5" s="2">
-        <f t="shared" ref="F5:F17" si="1">J5*H5</f>
+        <f t="shared" ref="F5" si="1">J5*H5</f>
         <v>36.800000400000002</v>
       </c>
       <c r="H5">
@@ -575,7 +581,7 @@
         <v>11</v>
       </c>
       <c r="F6" s="2">
-        <f t="shared" ref="F6:F17" si="2">SUM(J6:J7)-F7</f>
+        <f t="shared" ref="F6" si="2">SUM(J6:J7)-F7</f>
         <v>55.800000000000004</v>
       </c>
       <c r="H6">
@@ -602,7 +608,7 @@
         <v>11</v>
       </c>
       <c r="F7" s="2">
-        <f t="shared" ref="F7:F17" si="3">J7*H7</f>
+        <f t="shared" ref="F7" si="3">J7*H7</f>
         <v>37.199999999999996</v>
       </c>
       <c r="H7">
@@ -629,7 +635,7 @@
         <v>11</v>
       </c>
       <c r="F8" s="2">
-        <f t="shared" ref="F8:F17" si="4">SUM(J8:J9)-F9</f>
+        <f t="shared" ref="F8" si="4">SUM(J8:J9)-F9</f>
         <v>58.2000004</v>
       </c>
       <c r="H8">
@@ -656,7 +662,7 @@
         <v>11</v>
       </c>
       <c r="F9" s="2">
-        <f t="shared" ref="F9:F17" si="5">J9*H9</f>
+        <f t="shared" ref="F9" si="5">J9*H9</f>
         <v>38.7999996</v>
       </c>
       <c r="H9">
@@ -683,7 +689,7 @@
         <v>11</v>
       </c>
       <c r="F10" s="2">
-        <f t="shared" ref="F10:F17" si="6">SUM(J10:J11)-F11</f>
+        <f t="shared" ref="F10" si="6">SUM(J10:J11)-F11</f>
         <v>55.800000000000004</v>
       </c>
       <c r="H10">
@@ -710,7 +716,7 @@
         <v>11</v>
       </c>
       <c r="F11" s="2">
-        <f t="shared" ref="F11:F17" si="7">J11*H11</f>
+        <f t="shared" ref="F11" si="7">J11*H11</f>
         <v>37.199999999999996</v>
       </c>
       <c r="H11">
@@ -737,7 +743,7 @@
         <v>11</v>
       </c>
       <c r="F12" s="2">
-        <f t="shared" ref="F12:F17" si="8">SUM(J12:J13)-F13</f>
+        <f t="shared" ref="F12" si="8">SUM(J12:J13)-F13</f>
         <v>56.999999600000002</v>
       </c>
       <c r="H12">
@@ -764,7 +770,7 @@
         <v>11</v>
       </c>
       <c r="F13" s="2">
-        <f t="shared" ref="F13:F17" si="9">J13*H13</f>
+        <f t="shared" ref="F13" si="9">J13*H13</f>
         <v>38.000000399999998</v>
       </c>
       <c r="H13">
@@ -791,7 +797,7 @@
         <v>11</v>
       </c>
       <c r="F14" s="2">
-        <f t="shared" ref="F14:F17" si="10">SUM(J14:J15)-F15</f>
+        <f t="shared" ref="F14" si="10">SUM(J14:J15)-F15</f>
         <v>54</v>
       </c>
       <c r="H14">
@@ -818,7 +824,7 @@
         <v>11</v>
       </c>
       <c r="F15" s="2">
-        <f t="shared" ref="F15:F17" si="11">J15*H15</f>
+        <f t="shared" ref="F15" si="11">J15*H15</f>
         <v>36</v>
       </c>
       <c r="H15">
@@ -845,7 +851,7 @@
         <v>11</v>
       </c>
       <c r="F16" s="2">
-        <f t="shared" ref="F16:F17" si="12">SUM(J16:J17)-F17</f>
+        <f t="shared" ref="F16" si="12">SUM(J16:J17)-F17</f>
         <v>52.800000400000002</v>
       </c>
       <c r="H16">
@@ -904,12 +910,12 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="20.7109375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11.7109375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="22.7109375" bestFit="1" customWidth="1"/>
@@ -987,6 +993,110 @@
         <v>100</v>
       </c>
     </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D4" t="s">
+        <v>20</v>
+      </c>
+      <c r="E4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F4" t="s">
+        <v>17</v>
+      </c>
+      <c r="G4" t="s">
+        <v>16</v>
+      </c>
+      <c r="H4">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>21</v>
+      </c>
+      <c r="B5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G5" t="s">
+        <v>16</v>
+      </c>
+      <c r="H5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>21</v>
+      </c>
+      <c r="B6" t="s">
+        <v>23</v>
+      </c>
+      <c r="C6" t="s">
+        <v>25</v>
+      </c>
+      <c r="D6" t="s">
+        <v>20</v>
+      </c>
+      <c r="E6" t="s">
+        <v>8</v>
+      </c>
+      <c r="F6" t="s">
+        <v>17</v>
+      </c>
+      <c r="G6" t="s">
+        <v>16</v>
+      </c>
+      <c r="H6">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>21</v>
+      </c>
+      <c r="B7" t="s">
+        <v>23</v>
+      </c>
+      <c r="C7" t="s">
+        <v>26</v>
+      </c>
+      <c r="D7" t="s">
+        <v>20</v>
+      </c>
+      <c r="E7" t="s">
+        <v>8</v>
+      </c>
+      <c r="F7" t="s">
+        <v>17</v>
+      </c>
+      <c r="G7" t="s">
+        <v>16</v>
+      </c>
+      <c r="H7">
+        <v>100</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>